<commit_message>
Expand QA validation artifacts
- add validation and rule documents for auth, reading, community, and notifications

- update completed test case workbooks across Bible reading, community, and notifications

- revise bug report template and add completed community title/description report
</commit_message>
<xml_diff>
--- a/qa-docs/test-cases/Done/Me/Notifications/VerseByVerse_Notifications_Actions_Test_Cases.xlsx
+++ b/qa-docs/test-cases/Done/Me/Notifications/VerseByVerse_Notifications_Actions_Test_Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\versebyverse-quality-engineering\qa-docs\test-cases\Done\Notifications\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\versebyverse-quality-engineering\qa-docs\test-cases\Done\Me\Notifications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1852242D-8401-4D1B-AF79-127289AFAF76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3520F75F-2F94-433D-A034-16C6B2E1DB0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="243">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -857,6 +857,9 @@
   </si>
   <si>
     <t>Server-backed state persists and stale item does not reappear incorrectly</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
 </sst>
 </file>
@@ -1245,8 +1248,8 @@
     <col min="4" max="4" width="49.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="73.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.85546875" customWidth="1"/>
+    <col min="8" max="8" width="30.5703125" customWidth="1"/>
     <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
@@ -1302,7 +1305,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>28</v>
       </c>
@@ -1334,10 +1337,10 @@
         <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="165" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -1369,10 +1372,10 @@
         <v>12</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>40</v>
       </c>
@@ -1404,10 +1407,10 @@
         <v>12</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="195" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>46</v>
       </c>
@@ -1439,10 +1442,10 @@
         <v>18</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>51</v>
       </c>
@@ -1474,10 +1477,10 @@
         <v>18</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>56</v>
       </c>
@@ -1509,10 +1512,10 @@
         <v>19</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="165" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>62</v>
       </c>
@@ -1544,10 +1547,10 @@
         <v>17</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>67</v>
       </c>
@@ -1579,10 +1582,10 @@
         <v>18</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="165" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>73</v>
       </c>
@@ -1614,10 +1617,10 @@
         <v>12</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>78</v>
       </c>
@@ -1649,10 +1652,10 @@
         <v>12</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>83</v>
       </c>
@@ -1684,10 +1687,10 @@
         <v>12</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>88</v>
       </c>
@@ -1719,10 +1722,10 @@
         <v>18</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>93</v>
       </c>
@@ -1754,10 +1757,10 @@
         <v>12</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>99</v>
       </c>
@@ -1789,10 +1792,10 @@
         <v>12</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>105</v>
       </c>
@@ -1824,10 +1827,10 @@
         <v>12</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>109</v>
       </c>
@@ -1859,10 +1862,10 @@
         <v>19</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>113</v>
       </c>
@@ -1894,10 +1897,10 @@
         <v>18</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>118</v>
       </c>
@@ -1929,10 +1932,10 @@
         <v>12</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>124</v>
       </c>
@@ -1964,10 +1967,10 @@
         <v>12</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>129</v>
       </c>
@@ -1999,10 +2002,10 @@
         <v>12</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>134</v>
       </c>
@@ -2034,10 +2037,10 @@
         <v>18</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>140</v>
       </c>
@@ -2069,10 +2072,10 @@
         <v>12</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="105" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>145</v>
       </c>
@@ -2104,10 +2107,10 @@
         <v>12</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>151</v>
       </c>
@@ -2139,10 +2142,10 @@
         <v>18</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>156</v>
       </c>
@@ -2174,10 +2177,10 @@
         <v>19</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>161</v>
       </c>
@@ -2209,7 +2212,7 @@
         <v>12</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>13</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="60" x14ac:dyDescent="0.25">
@@ -2247,7 +2250,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="210" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>172</v>
       </c>
@@ -2279,10 +2282,10 @@
         <v>12</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>178</v>
       </c>
@@ -2314,10 +2317,10 @@
         <v>12</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>182</v>
       </c>
@@ -2349,10 +2352,10 @@
         <v>12</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>188</v>
       </c>
@@ -2384,10 +2387,10 @@
         <v>12</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>192</v>
       </c>
@@ -2419,10 +2422,10 @@
         <v>19</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="135" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>198</v>
       </c>
@@ -2454,10 +2457,10 @@
         <v>18</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="195" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>203</v>
       </c>
@@ -2489,10 +2492,10 @@
         <v>18</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="180" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>209</v>
       </c>
@@ -2524,10 +2527,10 @@
         <v>17</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>214</v>
       </c>
@@ -2559,10 +2562,10 @@
         <v>14</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>220</v>
       </c>
@@ -2594,10 +2597,10 @@
         <v>12</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>226</v>
       </c>
@@ -2629,10 +2632,10 @@
         <v>19</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="120" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>231</v>
       </c>
@@ -2664,10 +2667,10 @@
         <v>19</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>236</v>
       </c>
@@ -2699,7 +2702,7 @@
         <v>19</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>13</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -2707,6 +2710,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K1048576" xr:uid="{9FD3C16F-E8BF-4A96-B04F-25AFE96B577F}">
+      <formula1>"Passed,Failed,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>